<commit_message>
Fixed issues with density order
</commit_message>
<xml_diff>
--- a/Data/2019_F013B4_CO_PIT/2019_F013B4_CO_PIT_CropCanopy.xlsx
+++ b/Data/2019_F013B4_CO_PIT/2019_F013B4_CO_PIT_CropCanopy.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\mnt\Data1\USDA-ALARC\GIS\PDI project\cottondata\Data\2019_F013B4_CO_PIT\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{43A57FF7-6E04-4EEC-A9D3-45FAF5FD2B4D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{58C452B9-BFBB-430A-9CE4-27BA833A8243}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="16350" yWindow="-23415" windowWidth="17955" windowHeight="22395" firstSheet="3" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-1830" yWindow="-23190" windowWidth="17955" windowHeight="16800" firstSheet="2" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Height" sheetId="10" r:id="rId1"/>
@@ -9076,7 +9076,7 @@
       </c>
       <c r="I13" s="71"/>
       <c r="K13" s="68">
-        <f t="shared" ref="K13:K36" si="0">H13/2</f>
+        <f>H13/2</f>
         <v>3</v>
       </c>
       <c r="L13" s="70">
@@ -9111,7 +9111,7 @@
       </c>
       <c r="I14" s="71"/>
       <c r="K14" s="68">
-        <f t="shared" si="0"/>
+        <f t="shared" ref="K13:K36" si="0">H14/2</f>
         <v>3.5</v>
       </c>
       <c r="L14" s="70">
@@ -25746,7 +25746,7 @@
         <v>140</v>
       </c>
       <c r="B6" s="208">
-        <v>7.8740157480314963</v>
+        <v>7.4365704286964132</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.2">
@@ -25754,7 +25754,7 @@
         <v>141</v>
       </c>
       <c r="B7" s="208">
-        <v>6.1242344706911638</v>
+        <v>8.530183727034121</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.2">
@@ -25762,7 +25762,7 @@
         <v>142</v>
       </c>
       <c r="B8" s="208">
-        <v>8.530183727034121</v>
+        <v>6.1242344706911638</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.2">
@@ -25770,7 +25770,7 @@
         <v>143</v>
       </c>
       <c r="B9" s="208">
-        <v>7.4365704286964132</v>
+        <v>7.8740157480314963</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.2">
@@ -25810,7 +25810,7 @@
         <v>148</v>
       </c>
       <c r="B14" s="208">
-        <v>7.4365704286964132</v>
+        <v>5.6867891513560807</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.2">
@@ -25818,7 +25818,7 @@
         <v>149</v>
       </c>
       <c r="B15" s="208">
-        <v>6.99912510936133</v>
+        <v>5.4680664916885391</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.2">
@@ -25826,7 +25826,7 @@
         <v>150</v>
       </c>
       <c r="B16" s="208">
-        <v>5.4680664916885391</v>
+        <v>6.99912510936133</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.2">
@@ -25834,7 +25834,7 @@
         <v>151</v>
       </c>
       <c r="B17" s="208">
-        <v>5.6867891513560807</v>
+        <v>7.4365704286964132</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.2">
@@ -25874,7 +25874,7 @@
         <v>156</v>
       </c>
       <c r="B22" s="208">
-        <v>7.8740157480314963</v>
+        <v>7.4365704286964132</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.2">
@@ -25898,7 +25898,7 @@
         <v>159</v>
       </c>
       <c r="B25" s="208">
-        <v>7.4365704286964132</v>
+        <v>7.8740157480314963</v>
       </c>
     </row>
   </sheetData>

</xml_diff>